<commit_message>
Checkpoint 1 Lab 1
</commit_message>
<xml_diff>
--- a/simple_classification/ablation_results/ablation_results.xlsx
+++ b/simple_classification/ablation_results/ablation_results.xlsx
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S13"/>
+  <dimension ref="A1:S16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1447,12 +1447,218 @@
         <v>0</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Team Member 1</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>ReLU</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Adam</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Pyramid</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0.3080137369791667</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0.274782421875</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>0.9204</v>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>best val acc 0.9204 at epoch 10</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>0.9063666666666667</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>0.9204</v>
+      </c>
+      <c r="P14" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>ReLU</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>AdamW</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Pyramid</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>0.1199495361328125</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>0.1700195434570312</v>
+      </c>
+      <c r="K15" s="4" t="n">
+        <v>0.9601</v>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>best val acc 0.9629 at epoch 9</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>0.9684666666666667</v>
+      </c>
+      <c r="O15" s="4" t="n">
+        <v>0.9629</v>
+      </c>
+      <c r="P15" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q15" s="2" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n"/>
+      <c r="B16" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>ReLU</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>AdamP</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Pyramid</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>0.1263103434244792</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>0.1720289794921875</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>0.9585</v>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>best val acc 0.9653 at epoch 9</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>0.9674333333333334</v>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>0.9653</v>
+      </c>
+      <c r="P16" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q16" s="2" t="n">
+        <v>82.8</v>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A2:A4"/>
     <mergeCell ref="A11:A13"/>
-    <mergeCell ref="A2:A4"/>
     <mergeCell ref="A5:A7"/>
-    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="A14:A16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1464,7 +1670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G136"/>
+  <dimension ref="A1:G166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4609,6 +4815,696 @@
         <v>0.9552</v>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>13</v>
+      </c>
+      <c r="B137" t="n">
+        <v>1</v>
+      </c>
+      <c r="C137" t="n">
+        <v>1</v>
+      </c>
+      <c r="D137" t="n">
+        <v>0.39168134765625</v>
+      </c>
+      <c r="E137" t="n">
+        <v>0.8788166666666667</v>
+      </c>
+      <c r="F137" t="n">
+        <v>0.3001686279296875</v>
+      </c>
+      <c r="G137" t="n">
+        <v>0.9028</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>13</v>
+      </c>
+      <c r="B138" t="n">
+        <v>1</v>
+      </c>
+      <c r="C138" t="n">
+        <v>2</v>
+      </c>
+      <c r="D138" t="n">
+        <v>0.3252404296875</v>
+      </c>
+      <c r="E138" t="n">
+        <v>0.9011833333333333</v>
+      </c>
+      <c r="F138" t="n">
+        <v>0.2817805908203125</v>
+      </c>
+      <c r="G138" t="n">
+        <v>0.9081</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>13</v>
+      </c>
+      <c r="B139" t="n">
+        <v>1</v>
+      </c>
+      <c r="C139" t="n">
+        <v>3</v>
+      </c>
+      <c r="D139" t="n">
+        <v>0.310976953125</v>
+      </c>
+      <c r="E139" t="n">
+        <v>0.9047833333333334</v>
+      </c>
+      <c r="F139" t="n">
+        <v>0.320945703125</v>
+      </c>
+      <c r="G139" t="n">
+        <v>0.8984</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>13</v>
+      </c>
+      <c r="B140" t="n">
+        <v>1</v>
+      </c>
+      <c r="C140" t="n">
+        <v>4</v>
+      </c>
+      <c r="D140" t="n">
+        <v>0.3186113932291667</v>
+      </c>
+      <c r="E140" t="n">
+        <v>0.9019666666666667</v>
+      </c>
+      <c r="F140" t="n">
+        <v>0.2866072265625</v>
+      </c>
+      <c r="G140" t="n">
+        <v>0.9115</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>13</v>
+      </c>
+      <c r="B141" t="n">
+        <v>1</v>
+      </c>
+      <c r="C141" t="n">
+        <v>5</v>
+      </c>
+      <c r="D141" t="n">
+        <v>0.31438681640625</v>
+      </c>
+      <c r="E141" t="n">
+        <v>0.90325</v>
+      </c>
+      <c r="F141" t="n">
+        <v>0.33700654296875</v>
+      </c>
+      <c r="G141" t="n">
+        <v>0.8954</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>13</v>
+      </c>
+      <c r="B142" t="n">
+        <v>1</v>
+      </c>
+      <c r="C142" t="n">
+        <v>6</v>
+      </c>
+      <c r="D142" t="n">
+        <v>0.3143763020833333</v>
+      </c>
+      <c r="E142" t="n">
+        <v>0.9056666666666666</v>
+      </c>
+      <c r="F142" t="n">
+        <v>0.269556787109375</v>
+      </c>
+      <c r="G142" t="n">
+        <v>0.9187</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>13</v>
+      </c>
+      <c r="B143" t="n">
+        <v>1</v>
+      </c>
+      <c r="C143" t="n">
+        <v>7</v>
+      </c>
+      <c r="D143" t="n">
+        <v>0.3078590169270833</v>
+      </c>
+      <c r="E143" t="n">
+        <v>0.9069833333333334</v>
+      </c>
+      <c r="F143" t="n">
+        <v>0.2938723876953125</v>
+      </c>
+      <c r="G143" t="n">
+        <v>0.9055</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>13</v>
+      </c>
+      <c r="B144" t="n">
+        <v>1</v>
+      </c>
+      <c r="C144" t="n">
+        <v>8</v>
+      </c>
+      <c r="D144" t="n">
+        <v>0.3089641927083333</v>
+      </c>
+      <c r="E144" t="n">
+        <v>0.90605</v>
+      </c>
+      <c r="F144" t="n">
+        <v>0.310909228515625</v>
+      </c>
+      <c r="G144" t="n">
+        <v>0.9056</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>13</v>
+      </c>
+      <c r="B145" t="n">
+        <v>1</v>
+      </c>
+      <c r="C145" t="n">
+        <v>9</v>
+      </c>
+      <c r="D145" t="n">
+        <v>0.3018802734375</v>
+      </c>
+      <c r="E145" t="n">
+        <v>0.9091166666666667</v>
+      </c>
+      <c r="F145" t="n">
+        <v>0.290485107421875</v>
+      </c>
+      <c r="G145" t="n">
+        <v>0.905</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>13</v>
+      </c>
+      <c r="B146" t="n">
+        <v>1</v>
+      </c>
+      <c r="C146" t="n">
+        <v>10</v>
+      </c>
+      <c r="D146" t="n">
+        <v>0.3080137369791667</v>
+      </c>
+      <c r="E146" t="n">
+        <v>0.9063666666666667</v>
+      </c>
+      <c r="F146" t="n">
+        <v>0.274782421875</v>
+      </c>
+      <c r="G146" t="n">
+        <v>0.9204</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>14</v>
+      </c>
+      <c r="B147" t="n">
+        <v>1</v>
+      </c>
+      <c r="C147" t="n">
+        <v>1</v>
+      </c>
+      <c r="D147" t="n">
+        <v>0.2841398111979166</v>
+      </c>
+      <c r="E147" t="n">
+        <v>0.9159</v>
+      </c>
+      <c r="F147" t="n">
+        <v>0.2018853759765625</v>
+      </c>
+      <c r="G147" t="n">
+        <v>0.944</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>14</v>
+      </c>
+      <c r="B148" t="n">
+        <v>1</v>
+      </c>
+      <c r="C148" t="n">
+        <v>2</v>
+      </c>
+      <c r="D148" t="n">
+        <v>0.1870343098958333</v>
+      </c>
+      <c r="E148" t="n">
+        <v>0.9483833333333334</v>
+      </c>
+      <c r="F148" t="n">
+        <v>0.1700028442382812</v>
+      </c>
+      <c r="G148" t="n">
+        <v>0.9512</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>14</v>
+      </c>
+      <c r="B149" t="n">
+        <v>1</v>
+      </c>
+      <c r="C149" t="n">
+        <v>3</v>
+      </c>
+      <c r="D149" t="n">
+        <v>0.173436669921875</v>
+      </c>
+      <c r="E149" t="n">
+        <v>0.9531666666666667</v>
+      </c>
+      <c r="F149" t="n">
+        <v>0.1751197509765625</v>
+      </c>
+      <c r="G149" t="n">
+        <v>0.9525</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>14</v>
+      </c>
+      <c r="B150" t="n">
+        <v>1</v>
+      </c>
+      <c r="C150" t="n">
+        <v>4</v>
+      </c>
+      <c r="D150" t="n">
+        <v>0.1551606119791667</v>
+      </c>
+      <c r="E150" t="n">
+        <v>0.95835</v>
+      </c>
+      <c r="F150" t="n">
+        <v>0.21929697265625</v>
+      </c>
+      <c r="G150" t="n">
+        <v>0.9446</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>14</v>
+      </c>
+      <c r="B151" t="n">
+        <v>1</v>
+      </c>
+      <c r="C151" t="n">
+        <v>5</v>
+      </c>
+      <c r="D151" t="n">
+        <v>0.1517511393229167</v>
+      </c>
+      <c r="E151" t="n">
+        <v>0.9597</v>
+      </c>
+      <c r="F151" t="n">
+        <v>0.216556787109375</v>
+      </c>
+      <c r="G151" t="n">
+        <v>0.9466</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>14</v>
+      </c>
+      <c r="B152" t="n">
+        <v>1</v>
+      </c>
+      <c r="C152" t="n">
+        <v>6</v>
+      </c>
+      <c r="D152" t="n">
+        <v>0.1421634765625</v>
+      </c>
+      <c r="E152" t="n">
+        <v>0.9621166666666666</v>
+      </c>
+      <c r="F152" t="n">
+        <v>0.2119422607421875</v>
+      </c>
+      <c r="G152" t="n">
+        <v>0.9512</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>14</v>
+      </c>
+      <c r="B153" t="n">
+        <v>1</v>
+      </c>
+      <c r="C153" t="n">
+        <v>7</v>
+      </c>
+      <c r="D153" t="n">
+        <v>0.1392783854166667</v>
+      </c>
+      <c r="E153" t="n">
+        <v>0.9638666666666666</v>
+      </c>
+      <c r="F153" t="n">
+        <v>0.1938450073242187</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0.954</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>14</v>
+      </c>
+      <c r="B154" t="n">
+        <v>1</v>
+      </c>
+      <c r="C154" t="n">
+        <v>8</v>
+      </c>
+      <c r="D154" t="n">
+        <v>0.1359104654947917</v>
+      </c>
+      <c r="E154" t="n">
+        <v>0.9644</v>
+      </c>
+      <c r="F154" t="n">
+        <v>0.2060357421875</v>
+      </c>
+      <c r="G154" t="n">
+        <v>0.9529</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>14</v>
+      </c>
+      <c r="B155" t="n">
+        <v>1</v>
+      </c>
+      <c r="C155" t="n">
+        <v>9</v>
+      </c>
+      <c r="D155" t="n">
+        <v>0.1240345296223958</v>
+      </c>
+      <c r="E155" t="n">
+        <v>0.96735</v>
+      </c>
+      <c r="F155" t="n">
+        <v>0.15221357421875</v>
+      </c>
+      <c r="G155" t="n">
+        <v>0.9629</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>14</v>
+      </c>
+      <c r="B156" t="n">
+        <v>1</v>
+      </c>
+      <c r="C156" t="n">
+        <v>10</v>
+      </c>
+      <c r="D156" t="n">
+        <v>0.1199495361328125</v>
+      </c>
+      <c r="E156" t="n">
+        <v>0.9684666666666667</v>
+      </c>
+      <c r="F156" t="n">
+        <v>0.1700195434570312</v>
+      </c>
+      <c r="G156" t="n">
+        <v>0.9601</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>15</v>
+      </c>
+      <c r="B157" t="n">
+        <v>1</v>
+      </c>
+      <c r="C157" t="n">
+        <v>1</v>
+      </c>
+      <c r="D157" t="n">
+        <v>0.2745649739583333</v>
+      </c>
+      <c r="E157" t="n">
+        <v>0.9180333333333334</v>
+      </c>
+      <c r="F157" t="n">
+        <v>0.1887300048828125</v>
+      </c>
+      <c r="G157" t="n">
+        <v>0.9463</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>15</v>
+      </c>
+      <c r="B158" t="n">
+        <v>1</v>
+      </c>
+      <c r="C158" t="n">
+        <v>2</v>
+      </c>
+      <c r="D158" t="n">
+        <v>0.1877075032552083</v>
+      </c>
+      <c r="E158" t="n">
+        <v>0.9472166666666667</v>
+      </c>
+      <c r="F158" t="n">
+        <v>0.1545174072265625</v>
+      </c>
+      <c r="G158" t="n">
+        <v>0.9565</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>15</v>
+      </c>
+      <c r="B159" t="n">
+        <v>1</v>
+      </c>
+      <c r="C159" t="n">
+        <v>3</v>
+      </c>
+      <c r="D159" t="n">
+        <v>0.1687245768229167</v>
+      </c>
+      <c r="E159" t="n">
+        <v>0.9535666666666667</v>
+      </c>
+      <c r="F159" t="n">
+        <v>0.1616471801757813</v>
+      </c>
+      <c r="G159" t="n">
+        <v>0.9573</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>15</v>
+      </c>
+      <c r="B160" t="n">
+        <v>1</v>
+      </c>
+      <c r="C160" t="n">
+        <v>4</v>
+      </c>
+      <c r="D160" t="n">
+        <v>0.1545480305989583</v>
+      </c>
+      <c r="E160" t="n">
+        <v>0.9579333333333333</v>
+      </c>
+      <c r="F160" t="n">
+        <v>0.15520712890625</v>
+      </c>
+      <c r="G160" t="n">
+        <v>0.9586</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>15</v>
+      </c>
+      <c r="B161" t="n">
+        <v>1</v>
+      </c>
+      <c r="C161" t="n">
+        <v>5</v>
+      </c>
+      <c r="D161" t="n">
+        <v>0.145654345703125</v>
+      </c>
+      <c r="E161" t="n">
+        <v>0.9612166666666667</v>
+      </c>
+      <c r="F161" t="n">
+        <v>0.1826316650390625</v>
+      </c>
+      <c r="G161" t="n">
+        <v>0.9534</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>15</v>
+      </c>
+      <c r="B162" t="n">
+        <v>1</v>
+      </c>
+      <c r="C162" t="n">
+        <v>6</v>
+      </c>
+      <c r="D162" t="n">
+        <v>0.1387305826822917</v>
+      </c>
+      <c r="E162" t="n">
+        <v>0.9638833333333333</v>
+      </c>
+      <c r="F162" t="n">
+        <v>0.15875654296875</v>
+      </c>
+      <c r="G162" t="n">
+        <v>0.9603</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>15</v>
+      </c>
+      <c r="B163" t="n">
+        <v>1</v>
+      </c>
+      <c r="C163" t="n">
+        <v>7</v>
+      </c>
+      <c r="D163" t="n">
+        <v>0.1375716959635417</v>
+      </c>
+      <c r="E163" t="n">
+        <v>0.9637</v>
+      </c>
+      <c r="F163" t="n">
+        <v>0.170444921875</v>
+      </c>
+      <c r="G163" t="n">
+        <v>0.9608</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>15</v>
+      </c>
+      <c r="B164" t="n">
+        <v>1</v>
+      </c>
+      <c r="C164" t="n">
+        <v>8</v>
+      </c>
+      <c r="D164" t="n">
+        <v>0.14201455078125</v>
+      </c>
+      <c r="E164" t="n">
+        <v>0.9636333333333333</v>
+      </c>
+      <c r="F164" t="n">
+        <v>0.1620988525390625</v>
+      </c>
+      <c r="G164" t="n">
+        <v>0.958</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>15</v>
+      </c>
+      <c r="B165" t="n">
+        <v>1</v>
+      </c>
+      <c r="C165" t="n">
+        <v>9</v>
+      </c>
+      <c r="D165" t="n">
+        <v>0.1274048828125</v>
+      </c>
+      <c r="E165" t="n">
+        <v>0.96685</v>
+      </c>
+      <c r="F165" t="n">
+        <v>0.150406005859375</v>
+      </c>
+      <c r="G165" t="n">
+        <v>0.9653</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>15</v>
+      </c>
+      <c r="B166" t="n">
+        <v>1</v>
+      </c>
+      <c r="C166" t="n">
+        <v>10</v>
+      </c>
+      <c r="D166" t="n">
+        <v>0.1263103434244792</v>
+      </c>
+      <c r="E166" t="n">
+        <v>0.9674333333333334</v>
+      </c>
+      <c r="F166" t="n">
+        <v>0.1720289794921875</v>
+      </c>
+      <c r="G166" t="n">
+        <v>0.9585</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>